<commit_message>
Dashboard Update: ECN (SLH1-전체)
</commit_message>
<xml_diff>
--- a/data/ECN/ECN_STN_Master(SLH1).xlsx
+++ b/data/ECN/ECN_STN_Master(SLH1).xlsx
@@ -4557,7 +4557,11 @@
       </c>
       <c r="I77" s="11" t="inlineStr"/>
       <c r="J77" s="19" t="inlineStr"/>
-      <c r="K77" s="20" t="inlineStr"/>
+      <c r="K77" s="20" t="inlineStr">
+        <is>
+          <t>\\192.168.0.100\500 생산\550 국내CS\ECT&amp;STN\ECN SLH1-PP-260219-02(CCTV BRK 신규추가)</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="156.6" customHeight="1" s="21">
       <c r="B78" s="9" t="n">
@@ -4599,7 +4603,11 @@
       </c>
       <c r="I78" s="11" t="inlineStr"/>
       <c r="J78" s="19" t="inlineStr"/>
-      <c r="K78" s="20" t="inlineStr"/>
+      <c r="K78" s="20" t="inlineStr">
+        <is>
+          <t>\\192.168.0.100\500 생산\550 국내CS\ECT&amp;STN\ECN SLH1-PP-260225-01(Tray Flow Preciser Insert Pitch Fitting 추가)</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="52.2" customHeight="1" s="21">
       <c r="B79" s="9" t="n">
@@ -4676,7 +4684,11 @@
       </c>
       <c r="I80" s="11" t="inlineStr"/>
       <c r="J80" s="19" t="inlineStr"/>
-      <c r="K80" s="20" t="inlineStr"/>
+      <c r="K80" s="20" t="inlineStr">
+        <is>
+          <t>\\192.168.0.100\500 생산\550 국내CS\ECT&amp;STN\SLH1-PP-260305-01(SOCAMM HAND 공압 변경 및 필터 추가)</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="104.4" customHeight="1" s="21">
       <c r="B81" s="9" t="n">
@@ -4717,7 +4729,11 @@
       </c>
       <c r="I81" s="11" t="inlineStr"/>
       <c r="J81" s="19" t="inlineStr"/>
-      <c r="K81" s="20" t="inlineStr"/>
+      <c r="K81" s="20" t="inlineStr">
+        <is>
+          <t>\\192.168.0.100\500 생산\550 국내CS\ECT&amp;STN\ECN SLH1-PP-260227-01(후면부 Regulator Sensor 위치 개선)</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="243.6" customHeight="1" s="21">
       <c r="B82" s="9" t="n">
@@ -4760,7 +4776,11 @@
         </is>
       </c>
       <c r="I82" s="11" t="inlineStr"/>
-      <c r="J82" s="19" t="inlineStr"/>
+      <c r="J82" s="19" t="inlineStr">
+        <is>
+          <t>횡전개 완료.</t>
+        </is>
+      </c>
       <c r="K82" s="20" t="inlineStr">
         <is>
           <t>\\192.168.0.100\500 생산\550 국내CS\ECT&amp;STN\SLH1-PP-260306-01(LD Manual Port)</t>

</xml_diff>

<commit_message>
Add new ECN via Web
</commit_message>
<xml_diff>
--- a/data/ECN/ECN_STN_Master(SLH1).xlsx
+++ b/data/ECN/ECN_STN_Master(SLH1).xlsx
@@ -1429,7 +1429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K84"/>
+  <dimension ref="A2:K85"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.796875" defaultRowHeight="17.4"/>
   <cols>
     <col width="1.69921875" customWidth="1" style="16" min="1" max="1"/>
@@ -1770,9 +1770,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="n"/>
-      <c r="I8" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I8" s="11" t="n"/>
       <c r="J8" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -1818,9 +1816,7 @@
 -현재 SLH1 PC는 USB 3.0 PORT 로 구성되어있음</t>
         </is>
       </c>
-      <c r="I9" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I9" s="11" t="n"/>
       <c r="J9" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -1910,9 +1906,7 @@
           <t>-RD Tray Bending 개선, Rail 갈림현상 개선 -LPCAMM Tray Rail 갈림현상 개선</t>
         </is>
       </c>
-      <c r="I11" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I11" s="11" t="n"/>
       <c r="J11" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -1955,9 +1949,7 @@
           <t>SLH1 RD 최종 Insert(Latch 제거) 및 T-tray Bom Update</t>
         </is>
       </c>
-      <c r="I12" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I12" s="11" t="n"/>
       <c r="J12" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2095,9 +2087,7 @@
           <t>SLH1 RD 최종 INSERT 수량 정정(1ea&gt;16ea)</t>
         </is>
       </c>
-      <c r="I15" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I15" s="11" t="n"/>
       <c r="J15" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2139,9 +2129,7 @@
           <t>플러팅 기능 불가로 인한 가공 추가(선진행 요청)</t>
         </is>
       </c>
-      <c r="I16" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I16" s="11" t="n"/>
       <c r="J16" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2290,9 +2278,7 @@
  - LM과 조립 불가로 조립 기준 변경</t>
         </is>
       </c>
-      <c r="I19" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I19" s="11" t="n"/>
       <c r="J19" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2441,9 +2427,7 @@
 -도면 업데이트 및 부적합 사항 수정</t>
         </is>
       </c>
-      <c r="I22" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I22" s="11" t="n"/>
       <c r="J22" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2489,9 +2473,7 @@
 -신규 STOPPER 발주</t>
         </is>
       </c>
-      <c r="I23" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I23" s="11" t="n"/>
       <c r="J23" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2535,9 +2517,7 @@
 -Cover의 풀림 방지를 위한 너트 추가</t>
         </is>
       </c>
-      <c r="I24" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I24" s="11" t="n"/>
       <c r="J24" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2582,9 +2562,7 @@
 -크기 및 성능 동일 하며 CE 및 UL 인증 확인 완료.</t>
         </is>
       </c>
-      <c r="I25" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I25" s="11" t="n"/>
       <c r="J25" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2629,9 +2607,7 @@
 -1호기 때 조립기준과 달라져 배선 방향 변경으로 길이 변경하여 포설 필요</t>
         </is>
       </c>
-      <c r="I26" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I26" s="11" t="n"/>
       <c r="J26" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2682,9 +2658,7 @@
  - 간섭 미사용 구매품 폐기</t>
         </is>
       </c>
-      <c r="I27" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I27" s="11" t="n"/>
       <c r="J27" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2727,9 +2701,7 @@
 -제조팀 요청 공압 선 정리를 위한 홀 추가</t>
         </is>
       </c>
-      <c r="I28" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I28" s="11" t="n"/>
       <c r="J28" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2771,9 +2743,7 @@
           <t>잦은 파손으로 인한 재질 및 후처리 변경</t>
         </is>
       </c>
-      <c r="I29" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I29" s="11" t="n"/>
       <c r="J29" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2815,9 +2785,7 @@
           <t>고객사 요청 가공품 재질 및 후처리 변경</t>
         </is>
       </c>
-      <c r="I30" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I30" s="11" t="n"/>
       <c r="J30" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2863,9 +2831,7 @@
 -치수 누락으로 인한 도면 UPDATE (현품수정)</t>
         </is>
       </c>
-      <c r="I31" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I31" s="11" t="n"/>
       <c r="J31" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2907,9 +2873,7 @@
           <t>FITTING 연결부 크기 미일치로 인해 FITTING변경</t>
         </is>
       </c>
-      <c r="I32" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I32" s="11" t="n"/>
       <c r="J32" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2954,9 +2918,7 @@
 -모니터 회전의 어려움으로 인한 샤프트 길이 변경</t>
         </is>
       </c>
-      <c r="I33" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I33" s="11" t="n"/>
       <c r="J33" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -2999,9 +2961,7 @@
 -전장판 떨림 방지 개선</t>
         </is>
       </c>
-      <c r="I34" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I34" s="11" t="n"/>
       <c r="J34" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3050,9 +3010,7 @@
 -D컷 가공 추가</t>
         </is>
       </c>
-      <c r="I35" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I35" s="11" t="n"/>
       <c r="J35" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3098,9 +3056,7 @@
 -제조팀 요청 솔블록 추가</t>
         </is>
       </c>
-      <c r="I36" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I36" s="11" t="n"/>
       <c r="J36" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3145,9 +3101,7 @@
 -탭 위치 불량으로 인한 탭 추가</t>
         </is>
       </c>
-      <c r="I37" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I37" s="11" t="n"/>
       <c r="J37" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3191,9 +3145,7 @@
 -STACKER STOPPER 흐트러짐 개선 건(1호기 테스트 완료)</t>
         </is>
       </c>
-      <c r="I38" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I38" s="11" t="n"/>
       <c r="J38" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3238,9 +3190,7 @@
 -RAN CABLE 수량 누락</t>
         </is>
       </c>
-      <c r="I39" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I39" s="11" t="n"/>
       <c r="J39" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3333,9 +3283,7 @@
 -전장팀 요청 버튼 조작을 위한 REAR MONITER COVER의 여닫이 COVER 추가</t>
         </is>
       </c>
-      <c r="I41" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I41" s="11" t="n"/>
       <c r="J41" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3377,9 +3325,7 @@
           <t xml:space="preserve"> -SLH1 SOCAMM 전용 T-TRAY,MASK, PRECISER 등록 및 2호기 적용파트 발주 건(업체 JIG 지정 요청)</t>
         </is>
       </c>
-      <c r="I42" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I42" s="11" t="n"/>
       <c r="J42" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3425,9 +3371,7 @@
 ㄴ항목 11,13 수량 삭제 12,14 수량 변경 및 추가분 발주(SLH1-PP-251230-11 발주분 외 추가 발주) </t>
         </is>
       </c>
-      <c r="I43" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I43" s="11" t="n"/>
       <c r="J43" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3469,9 +3413,7 @@
           <t>도면 높이 치수 공차 추가 BOM UPDATE</t>
         </is>
       </c>
-      <c r="I44" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I44" s="11" t="n"/>
       <c r="J44" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3559,9 +3501,7 @@
           <t>제조팀 요청 마운트 탭 추가</t>
         </is>
       </c>
-      <c r="I46" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I46" s="11" t="n"/>
       <c r="J46" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3603,9 +3543,7 @@
           <t>VISION BRK 변경</t>
         </is>
       </c>
-      <c r="I47" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I47" s="11" t="n"/>
       <c r="J47" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3647,9 +3585,7 @@
           <t>FRAME 고정용 ANCHOR BRK 추가</t>
         </is>
       </c>
-      <c r="I48" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I48" s="11" t="n"/>
       <c r="J48" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3692,9 +3628,7 @@
 -EMS 황색 명판 삭제 요청(고객사 요청)</t>
         </is>
       </c>
-      <c r="I49" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I49" s="11" t="n"/>
       <c r="J49" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3738,9 +3672,7 @@
 -AF-BM 으로 변경하여 적용 예정</t>
         </is>
       </c>
-      <c r="I50" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I50" s="11" t="n"/>
       <c r="J50" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3782,9 +3714,7 @@
           <t>SLH1 SOCAMM INSC0-IB-06-0 : AD32CM INSERT 부품과 공용 사용/기존 도면 참조</t>
         </is>
       </c>
-      <c r="I51" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I51" s="11" t="n"/>
       <c r="J51" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3826,9 +3756,7 @@
           <t>LED 설치 BRK 추가</t>
         </is>
       </c>
-      <c r="I52" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I52" s="11" t="n"/>
       <c r="J52" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3870,9 +3798,7 @@
           <t>TRAY GUIDE BLOCK 길이 다르게 수정하여 TEST 진행</t>
         </is>
       </c>
-      <c r="I53" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I53" s="11" t="n"/>
       <c r="J53" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3920,9 +3846,7 @@
 -신규 블록 추가로 인한 홀 추가</t>
         </is>
       </c>
-      <c r="I54" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I54" s="11" t="n"/>
       <c r="J54" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -3970,9 +3894,7 @@
 -BUSH BLOCK TAP 양면 가공 추가</t>
         </is>
       </c>
-      <c r="I55" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I55" s="11" t="n"/>
       <c r="J55" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4018,9 +3940,7 @@
           <t>장비 제작 간 케이블 하네스 불합리 및 누락 케이블 추가 업데이트 및 구매</t>
         </is>
       </c>
-      <c r="I56" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I56" s="11" t="n"/>
       <c r="J56" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4063,9 +3983,7 @@
 -제조팀 요청 간섭 및 조립 편의성을 위한 홀 타입 변경</t>
         </is>
       </c>
-      <c r="I57" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I57" s="11" t="n"/>
       <c r="J57" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4111,9 +4029,7 @@
           <t>SOCAMM HAND VISION BRK 변경으로 인한 설계 변경</t>
         </is>
       </c>
-      <c r="I58" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I58" s="11" t="n"/>
       <c r="J58" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4157,9 +4073,7 @@
 -신규 브라켓 추가로 인한 블록 TAP 추가</t>
         </is>
       </c>
-      <c r="I59" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I59" s="11" t="n"/>
       <c r="J59" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4205,9 +4119,7 @@
           <t>장비 제작 간 케이블 하네스 불합리 및 누락 케이블 추가 업데이트</t>
         </is>
       </c>
-      <c r="I60" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I60" s="11" t="n"/>
       <c r="J60" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4249,9 +4161,7 @@
           <t>장비 제작 간 케이블 하네스 불합리 및 누락 케이블 추가 업데이트</t>
         </is>
       </c>
-      <c r="I61" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I61" s="11" t="n"/>
       <c r="J61" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4344,9 +4254,7 @@
 -ALIGN SHAFT 위치 조절 불가로 인한 블록 형상 변경</t>
         </is>
       </c>
-      <c r="I63" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I63" s="11" t="n"/>
       <c r="J63" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4392,9 +4300,7 @@
           <t>고객사 요구사항에 대응되는 PAD로 변경(마크리스 특수코팅 추가)</t>
         </is>
       </c>
-      <c r="I64" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I64" s="11" t="n"/>
       <c r="J64" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4443,9 +4349,7 @@
 -고객사 요청 재질 변경</t>
         </is>
       </c>
-      <c r="I65" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I65" s="11" t="n"/>
       <c r="J65" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4493,9 +4397,7 @@
 -케이블과 간섭으로 인한 가공 추가</t>
         </is>
       </c>
-      <c r="I66" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I66" s="11" t="n"/>
       <c r="J66" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4542,9 +4444,7 @@
 -TRAY 진입 불가로 인한 가공품 두께 변경</t>
         </is>
       </c>
-      <c r="I67" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I67" s="11" t="n"/>
       <c r="J67" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4592,9 +4492,7 @@
 -하위 파트 REV 변경에 따른 REV 변경, 조립 위치 변경</t>
         </is>
       </c>
-      <c r="I68" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I68" s="11" t="n"/>
       <c r="J68" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4640,9 +4538,7 @@
 -SPRING 결합 위치 변경 및 OPEN 각도 조정을 위한 형상 변경</t>
         </is>
       </c>
-      <c r="I69" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I69" s="11" t="n"/>
       <c r="J69" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4685,9 +4581,7 @@
 -가공업체 요청 라운드 값 변경, 표면 저항값 삭제</t>
         </is>
       </c>
-      <c r="I70" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I70" s="11" t="n"/>
       <c r="J70" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4735,9 +4629,7 @@
 -STACKER MANUAL PORT 롤러 간섭으로 인한 가공 추가</t>
         </is>
       </c>
-      <c r="I71" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I71" s="11" t="n"/>
       <c r="J71" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4789,9 +4681,7 @@
 -구매팀 요청 CCTV 세트화 해제로 인한 추가 발주</t>
         </is>
       </c>
-      <c r="I72" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I72" s="11" t="n"/>
       <c r="J72" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4841,9 +4731,7 @@
 -SHAFT 사이의 틈이 좁아 휨 이슈로 인한 가공 추가</t>
         </is>
       </c>
-      <c r="I73" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I73" s="11" t="n"/>
       <c r="J73" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4889,9 +4777,7 @@
           <t>BOM 수량 MISS 건 BOM UPDATE</t>
         </is>
       </c>
-      <c r="I74" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I74" s="11" t="n"/>
       <c r="J74" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4933,9 +4819,7 @@
           <t>고객사 요청 판넬 모서리 보호대 추가</t>
         </is>
       </c>
-      <c r="I75" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I75" s="11" t="n"/>
       <c r="J75" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -4981,9 +4865,7 @@
           <t>CCTV 브라켓 신규 추가</t>
         </is>
       </c>
-      <c r="I76" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I76" s="11" t="n"/>
       <c r="J76" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -5029,9 +4911,7 @@
           <t>장비제작 간 케이블 하네스 불합리 및 누락 케이블 추가 업데이트</t>
         </is>
       </c>
-      <c r="I77" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I77" s="11" t="n"/>
       <c r="J77" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -5081,9 +4961,7 @@
 -신규 브라켓 추가로 인한 기존 브라켓 및 ROLLER 4EA 폐기</t>
         </is>
       </c>
-      <c r="I78" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I78" s="11" t="n"/>
       <c r="J78" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -5130,9 +5008,7 @@
 -설계 MISS로 인한 변경 진행(긴급, 고객 검수 다음주 진행)</t>
         </is>
       </c>
-      <c r="I79" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I79" s="11" t="n"/>
       <c r="J79" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -5174,9 +5050,7 @@
           <t>고객사 요청 SOCAMM HAND GRIP의 공압을 최소로 가져가기 위한 브라켓 설계 변경 및 SPACER, AIR FILTER 추가</t>
         </is>
       </c>
-      <c r="I80" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I80" s="11" t="n"/>
       <c r="J80" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -5225,9 +5099,7 @@
 -SOCAMM PRECISER CONVERSION 체크 브러캣 추가</t>
         </is>
       </c>
-      <c r="I81" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I81" s="11" t="n"/>
       <c r="J81" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -5279,9 +5151,7 @@
 -SOCAMM STACKER ALIGN SHAFT 처짐으로 인한 BRACKET,LM GUIDE 추가</t>
         </is>
       </c>
-      <c r="I82" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I82" s="11" t="n"/>
       <c r="J82" s="19" t="inlineStr">
         <is>
           <t>횡전개 완료.</t>
@@ -5331,9 +5201,7 @@
 -상위 ASSY 도면 업데이트</t>
         </is>
       </c>
-      <c r="I83" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I83" s="11" t="n"/>
       <c r="J83" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
@@ -5376,15 +5244,62 @@
 -STACKER REJECK BOTTOM 컨베이어 STOP을 위한 센서 홀 없음</t>
         </is>
       </c>
-      <c r="I84" s="11" t="n">
-        <v/>
-      </c>
+      <c r="I84" s="11" t="n"/>
       <c r="J84" s="19" t="inlineStr">
         <is>
           <t>완료.</t>
         </is>
       </c>
       <c r="K84" s="20" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>기구설계팀</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>손희주</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SLH1 </t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>SLH1-PP-260506-01</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>STACKER REJECT ALIGN GUIDE 기능 불가로 인한 개선 건</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>-STACKER REJECT ALIGN GUIDE BRACKET 사이의 폭이 C-TRAY의 폭 보다 넓어 매번 같은 위치로 투입 불가  / -STACKER REJECT ALIGN GUIDE BRACKET의 SIZE 축소, 두 파트로 나누어 조절 포인트 추가</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>대기</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>\\192.168.0.100\500 생산\550 국내CS\ECN&amp;STN\SLH1-PP-260506-01.pdf</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>